<commit_message>
Add discarded pattern records
</commit_message>
<xml_diff>
--- a/Data/RQ2_Samples/Case_Judgments.xlsx
+++ b/Data/RQ2_Samples/Case_Judgments.xlsx
@@ -14,6 +14,7 @@
   </bookViews>
   <sheets>
     <sheet name="Case Judgments" sheetId="1" r:id="rId1"/>
+    <sheet name="Discarded Patterns" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -287,7 +288,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="@"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -305,8 +309,23 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF24313D"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -318,8 +337,31 @@
         <fgColor rgb="FF243B53"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF243B53"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -328,10 +370,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -341,6 +384,38 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2189,4 +2264,61 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="29" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="60" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="76" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="10" t="str">
+        <x:v>Configuration / Element</x:v>
+      </x:c>
+      <x:c r="B1" s="10" t="str">
+        <x:v>Discarded characterization</x:v>
+      </x:c>
+      <x:c r="C1" s="10" t="str">
+        <x:v>Non-matches / Reviewed</x:v>
+      </x:c>
+      <x:c r="D1" s="10" t="str">
+        <x:v>Non-matching cases</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="62" customHeight="1">
+      <x:c r="A2" s="11" t="str">
+        <x:v>Chained / Test Goal</x:v>
+      </x:c>
+      <x:c r="B2" s="11" t="str">
+        <x:v>Formulates the verification purpose within the scope defined by the extracted targets.</x:v>
+      </x:c>
+      <x:c r="C2" s="14" t="str">
+        <x:v>7/10</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="str">
+        <x:v>US13_2, teste2e.cy_1, xhr.cy_1, sample.test_3_4, vlSpecEditor.test, app.test_1, dog.test_2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="62" customHeight="1">
+      <x:c r="A3" s="7" t="str">
+        <x:v>DeepSeek 7B / Test Objects</x:v>
+      </x:c>
+      <x:c r="B3" s="7" t="str">
+        <x:v>More often focuses on local metadata entities and internal structures.</x:v>
+      </x:c>
+      <x:c r="C3" s="15" t="str">
+        <x:v>8/10</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="str">
+        <x:v>US13_2, teste2e.cy_1, xhr.cy_1, sample.test_3_4, ContinentRepositoryTest, soak, app.test_1, dog.test_2</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>